<commit_message>
zone_master.xlsx file updated. zone_layouts.md updated.
</commit_message>
<xml_diff>
--- a/layouts/master_layout/ZONE_MASTER.xlsx
+++ b/layouts/master_layout/ZONE_MASTER.xlsx
@@ -639,7 +639,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>P&amp;T1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>PACKAGING_TEST</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -736,12 +736,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>M14</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>FRONT_END_FAB</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -843,17 +843,17 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>DRAM</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>HBM</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>M16</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>FRONT_END_FAB</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1057,17 +1057,17 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>DRAM</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>P&amp;T5</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>PACKAGING_TEST</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1164,17 +1164,17 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HBM</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>M11_M12</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>FRONT_END_FAB</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1485,17 +1485,17 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>NAND</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>P&amp;T3</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>PACKAGING_TEST</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1592,17 +1592,17 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>NAND</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1704,12 +1704,12 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>DRAM</t>
+          <t>NAND</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1846,7 +1846,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2993,7 +2993,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -3130,7 +3130,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3528,7 +3528,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3742,7 +3742,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -3986,7 +3986,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4272,12 +4272,12 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>DRAM</t>
+          <t>DRAM_NAND</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -4307,7 +4307,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4379,12 +4379,12 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>MIXED</t>
+          <t>DRAM_NAND_LOGIC</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4461,7 +4461,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>V2</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -4471,7 +4471,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>FRONT_END_FAB</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -4481,17 +4481,17 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>LOGIC_DRAM_NAND</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -4521,7 +4521,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4568,7 +4568,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>FRONT_END_FAB</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -4588,17 +4588,17 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>DRAM_NAND_LOGIC</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4675,17 +4675,17 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>SSE_PTK_MX_001</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>FRONT_END_FAB</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -4695,17 +4695,17 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HBM_DRAM_NAND</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -4735,7 +4735,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4842,7 +4842,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5056,7 +5056,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5377,7 +5377,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5484,7 +5484,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5591,7 +5591,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5698,7 +5698,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5805,7 +5805,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -5912,7 +5912,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>2026-10-22 03:53</t>
+          <t>2026-10-26 00:53</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">

</xml_diff>

<commit_message>
zone_boundary_master.kml: finalized zone_master.xlsx: finalized
</commit_message>
<xml_diff>
--- a/layouts/master_layout/ZONE_MASTER.xlsx
+++ b/layouts/master_layout/ZONE_MASTER.xlsx
@@ -639,7 +639,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1846,7 +1846,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2993,7 +2993,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -3130,7 +3130,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3528,7 +3528,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3742,7 +3742,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -3986,7 +3986,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4277,7 +4277,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -4307,7 +4307,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4384,7 +4384,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -4521,7 +4521,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4598,7 +4598,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>HIGHLY_ASSOC</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -4735,7 +4735,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4842,7 +4842,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5056,7 +5056,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5377,7 +5377,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5484,7 +5484,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5591,7 +5591,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5698,7 +5698,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5805,7 +5805,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -5912,7 +5912,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -6340,7 +6340,7 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -6387,7 +6387,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -6447,12 +6447,12 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>127.1147064723468,36.8410849791771,0 127.1155832122999,36.84273177232313,0 127.1119293939781,36.84391880969204,0 127.1114404208229,36.84295845417474,0 127.1123291067114,36.84268048454407,0 127.111978484289,36.84196861807236,0 127.1147064723468,36.8410849791771,0</t>
+          <t>127.1176281814552,36.84023049977989,0 127.1184571394864,36.84184667940427,0 127.1173202441774,36.84220414477994,0 127.1164998825625,36.84060921633508,0 127.1176281814552,36.84023049977989,0</t>
         </is>
       </c>
     </row>
@@ -6554,7 +6554,7 @@
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>2026-10-27 02:30</t>
+          <t>2026-10-27 02:37</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">

</xml_diff>

<commit_message>
Set campus-division zone_type to NULL, make SSE_PTK_MX_01 an OAE zone
- Campus-division rows: zone_type CD -> NULL (12 zones); zone_code keeps CD
  and the build and validator find campus divisions by zone_code.
- SSE_PTK_MX_01 (P4) -> SSE_PTK_OAE_01, same record_id SSE_PTK_005; unit
  fields NULL, product MIXED. MX_HANDLING removed; TRANSFORM allows EX -> OAE.
- Build ZONE_OWNER_CARD_MASTER (12 current CD zones) and ZONE_OWNER_FT_MASTER
  (all 53 zones with effective dates), replacing ZONE_OWNER_MASTER.
- Rebuild ZONE_MASTER.xlsx and ZONE_BOUNDARY_MASTER.zip; update ZONE_LAYOUTS.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/layouts/master_layout/ZONE_MASTER.xlsx
+++ b/layouts/master_layout/ZONE_MASTER.xlsx
@@ -3,24 +3,25 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-8340" yWindow="-28800" windowWidth="51200" windowHeight="28800" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="ZONE_MASTER" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="ZONE_LINEAGE_MASTER" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ZONE_BOUNDARY_MASTER" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="FT_LIST_ZONE" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ZONE_OWNER_MASTER" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ZONE_OWNER_CARD_MASTER" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ZONE_OWNER_FT_MASTER" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ZONE_BOUNDARY_MASTER" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FT_LIST_ZONE" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,17 +31,23 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="16"/>
+      <color rgb="FF0070C0"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="18"/>
-      <scheme val="minor"/>
+      <color rgb="FF0070C0"/>
+      <sz val="16"/>
     </font>
   </fonts>
   <fills count="3">
@@ -53,7 +60,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -69,15 +75,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -224,6 +232,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -258,6 +267,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -292,20 +302,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -427,7 +433,46 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -461,111 +506,111 @@
     <col width="18.83203125" customWidth="1" min="18" max="18"/>
     <col width="27.6640625" customWidth="1" min="19" max="19"/>
     <col width="21.83203125" customWidth="1" min="20" max="20"/>
-    <col width="255.83203125" customWidth="1" min="21" max="21"/>
+    <col width="42.1640625" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>record_id</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>zone_code</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>company_name_en</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>security_code</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>campus_name</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>campus_code</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>campus_address</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>production_unit_name</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>production_unit_code</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>production_unit_type</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>zone_type</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>zone_type_confidence</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>primary_product_association</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>product_association_confidence</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>effective_from</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>effective_to</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>pit_available_from</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>pit_available_to</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>imagery_acquired_date</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>record_created_at</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>polygon</t>
         </is>
@@ -669,7 +714,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -776,7 +821,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -883,7 +928,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -990,7 +1035,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1097,7 +1142,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1204,7 +1249,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1311,7 +1356,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1371,9 +1416,9 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>CD</t>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1418,7 +1463,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1525,7 +1570,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1632,7 +1677,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1739,7 +1784,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1846,7 +1891,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1953,7 +1998,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -2060,7 +2105,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2167,7 +2212,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2227,9 +2272,9 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>CD</t>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -2274,7 +2319,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2334,9 +2379,9 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>CD</t>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2381,7 +2426,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2441,9 +2486,9 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>CD</t>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2488,7 +2533,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2548,9 +2593,9 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>CD</t>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2595,7 +2640,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2655,9 +2700,9 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>CD</t>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2702,7 +2747,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2809,7 +2854,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2869,9 +2914,9 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>CD</t>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2916,7 +2961,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -3023,7 +3068,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3130,7 +3175,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3237,7 +3282,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3297,9 +3342,9 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>CD</t>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -3344,7 +3389,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3451,7 +3496,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3558,7 +3603,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3665,7 +3710,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3772,7 +3817,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3879,7 +3924,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3986,7 +4031,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4093,7 +4138,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4153,9 +4198,9 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>CD</t>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -4200,7 +4245,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4307,7 +4352,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4414,7 +4459,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4521,7 +4566,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4628,7 +4673,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4643,9 +4688,9 @@
           <t>SSE_PTK_005</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>SSE_PTK_MX_01</t>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>SSE_PTK_OAE_01</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4673,24 +4718,24 @@
           <t>114, Samseong-ro, Pyeongtaek-si, Gyeonggi-do (17786)</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>SSE_PTK_MX_001</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>FRONT_END_FAB</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>MX</t>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>OAE</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -4698,9 +4743,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>HBM_DRAM_NAND</t>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>MIXED</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -4735,7 +4780,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4842,7 +4887,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4949,7 +4994,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5056,7 +5101,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5163,7 +5208,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5270,7 +5315,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5377,7 +5422,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5437,9 +5482,9 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>CD</t>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -5484,7 +5529,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5544,9 +5589,9 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>CD</t>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -5591,7 +5636,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5698,7 +5743,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5805,7 +5850,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -5912,7 +5957,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -6019,7 +6064,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -6126,7 +6171,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -6186,9 +6231,9 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>CD</t>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -6233,7 +6278,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>2026-10-26 00:53</t>
+          <t>2026-10-27 01:19</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -6256,47 +6301,48 @@
   <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="13.83203125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="22.83203125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="20.33203125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="22.83203125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="16" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="24.5" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="21.1640625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="13.83203125" customWidth="1" min="1" max="1"/>
+    <col width="22.83203125" customWidth="1" min="2" max="2"/>
+    <col width="20.33203125" customWidth="1" min="3" max="3"/>
+    <col width="22.83203125" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="24.5" customWidth="1" min="6" max="6"/>
+    <col width="21.1640625" customWidth="1" min="7" max="7"/>
+    <col width="13.5" customWidth="1" min="8" max="24"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customFormat="1" customHeight="1" s="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>lineage_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>parent_record_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>child_record_id</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>relationship_type</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>effective_at</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>pit_available_from</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>pit_available_to</t>
         </is>
@@ -6558,6 +6604,181 @@
       <c r="G8" t="inlineStr">
         <is>
           <t>NULL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14.6640625" customWidth="1" min="1" max="1"/>
+    <col width="42.1640625" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="21" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>zone_code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SKH_ICH_CD_01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>127.4792908753239,37.25468493538708,0 127.4786741753453,37.25444924351592,0 127.4772528388912,37.25395564829143,0 127.4767669938143,37.25346355087292,0 127.4760965089844,37.2524207558015,0 127.4754361562875,37.25013297475242,0 127.4755263691511,37.24998272523067,0 127.4761815390762,37.24996768272318,0 127.4762852154837,37.2491772417373,0 127.4766660853097,37.24888413057281,0 127.4770365177835,37.24820942523911,0 127.4770129777922,37.24630386888008,0 127.4783445671774,37.24652078460043,0 127.4794165116467,37.24653038307022,0 127.4797541563503,37.24665384241348,0 127.4823052038301,37.24663760873185,0 127.4826221319934,37.24669367528909,0 127.4826199787886,37.24693028697282,0 127.4839309344984,37.24692849021164,0 127.4851389162666,37.24673774714464,0 127.4857037675637,37.24680396813539,0 127.4864819820665,37.24661121408833,0 127.4878377799842,37.24645368922819,0 127.4878622737257,37.24765802504077,0 127.4887095942767,37.24765852211029,0 127.4887172526127,37.24795890179502,0 127.4909139624968,37.24894757882421,0 127.4906904523238,37.24976641620731,0 127.4901601862512,37.25102843554481,0 127.4886617641543,37.25291476424426,0 127.4869696609773,37.25478884788198,0 127.4861705759206,37.25455007950498,0 127.4853195412984,37.25499405132114,0 127.4845027267799,37.25543761273426,0 127.4841281940734,37.25522463987738,0 127.4797279161993,37.25522397442263,0 127.4792908753239,37.25468493538708,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_CD_01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>127.4275297354299,36.65233372032262,0 127.4263057730211,36.65185408401877,0 127.4262935535888,36.65122515869427,0 127.4275256456034,36.65122133567544,0 127.4275201588123,36.64961054877304,0 127.4312464208049,36.64960916510265,0 127.4312470904888,36.64952629302427,0 127.4351002158643,36.64950044912582,0 127.435166824625,36.65359448360476,0 127.432862488071,36.65359823906715,0 127.4316649289962,36.65337928541467,0 127.4308305599157,36.65296363320886,0 127.4288246715552,36.65263268339037,0 127.4275297354299,36.65233372032262,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_CD_02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>127.4260432086972,36.65176170137349,0 127.4248531681613,36.65127349565639,0 127.4237537290272,36.65063059263603,0 127.4234767236715,36.65009942631145,0 127.4232265303528,36.64810824397203,0 127.4247733956071,36.64798844700252,0 127.4255746104511,36.64780770534722,0 127.4260432086972,36.65176170137349,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_CD_03</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>127.4317942851492,36.64759990559355,0 127.4275552059397,36.64762560914508,0 127.4274902029552,36.64587102656827,0 127.4294903446101,36.64501362772035,0 127.4317576818901,36.64466362443578,0 127.4317942851492,36.64759990559355,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_CD_04</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>127.4292728903329,36.65737585583252,0 127.4273960610812,36.65679768320321,0 127.4282675369856,36.6554496975609,0 127.4284050618595,36.65469966598357,0 127.4282398485941,36.65293596566627,0 127.4304563399528,36.65307861551903,0 127.4316145244017,36.65366103982478,0 127.4326545386969,36.65382547046487,0 127.4350916090492,36.65392998807685,0 127.4352735323493,36.65785267344271,0 127.4292728903329,36.65737585583252,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_CD_05</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>127.4243211838829,36.6632598487266,0 127.424011351887,36.65991970480072,0 127.4229741451245,36.65607422634487,0 127.4244942262898,36.65536905146344,0 127.4257468499067,36.65639926020843,0 127.4267895578782,36.65700917768972,0 127.4282817570568,36.65755430873217,0 127.4297234332019,36.6578268621073,0 127.4353019051501,36.65834157696911,0 127.4356995447989,36.66481575781614,0 127.433912758689,36.66409712773648,0 127.4282703545717,36.66376686338138,0 127.4243211838829,36.6632598487266,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SKH_YIN_CD_01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>127.3165991989156,37.15980583693546,0 127.3128009723789,37.14835919575778,0 127.311076347084,37.14547863343643,0 127.3102408044489,37.14303692870982,0 127.3208615727544,37.14061591456515,0 127.3220561267111,37.1417979786553,0 127.3247735631805,37.14850423312373,0 127.324982600008,37.15064631017324,0 127.3266053447182,37.15485998175167,0 127.3279031725835,37.15572439755587,0 127.328670071381,37.15778146758801,0 127.3183489938163,37.16020717025311,0 127.3165991989156,37.15980583693546,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SSE_GHG_CD_01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>127.083461691631,37.22989691093171,0 127.083042227891,37.22951575495898,0 127.0829522524925,37.22638055251159,0 127.0844632219606,37.22638940835161,0 127.0844822059877,37.22570474903128,0 127.0887076667388,37.22570338865468,0 127.089052454588,37.22595566548927,0 127.089026146627,37.22718421375711,0 127.0895887134091,37.22719165032877,0 127.0891868539899,37.22816160042641,0 127.0887849945707,37.22913155052407,0 127.0880244523491,37.22991225379975,0 127.083461691631,37.22989691093171,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SSE_HWA_CD_01</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>127.0604088113161,37.22131882984505,0 127.0615807830927,37.22041598662344,0 127.0630934084169,37.21750233768811,0 127.0634913563929,37.21689581411416,0 127.0648657301476,37.21768520734643,0 127.0645369158691,37.21804783507638,0 127.0649234166045,37.21824765192734,0 127.0647277837963,37.21847858521478,0 127.0662831589923,37.21938670995086,0 127.06664594273,37.21885044069479,0 127.0670258100668,37.2180123534205,0 127.0670166258656,37.21713827335517,0 127.0674025178071,37.2155538216505,0 127.0667276391382,37.21500375126403,0 127.0655461123071,37.2149879687613,0 127.0648952488986,37.21559495354837,0 127.0634374596184,37.21535848732494,0 127.0642118961364,37.2123743909837,0 127.0651782203331,37.21208702120425,0 127.0677572511424,37.21194828414612,0 127.0705415107046,37.21031086343675,0 127.0728251102545,37.2120405976308,0 127.0781759625584,37.2149215297925,0 127.0774851858635,37.21729625905924,0 127.076012950966,37.22023406713998,0 127.0730025425854,37.21894843108969,0 127.0718544566005,37.21858037365727,0 127.0695738141374,37.21824888550046,0 127.0690641747031,37.21989668149228,0 127.0678519558422,37.21967489336973,0 127.0678501450078,37.21927789628356,0 127.0668359627562,37.21905080170365,0 127.0665419684045,37.21945597062771,0 127.065715293898,37.221067494351,0 127.0650135511269,37.22274342329509,0 127.0649907298155,37.22317211827212,0 127.0646802506171,37.2231710187238,0 127.0643725197762,37.22354909864806,0 127.0632761594175,37.22369709565476,0 127.0619533378606,37.22289446612139,0 127.0604088113161,37.22131882984505,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SSE_PTK_CD_01</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>127.054266060945,37.03416232535104,0 127.0543122205523,37.02756427257659,0 127.0681249737192,37.0275595754502,0 127.0674879668247,37.03507496714188,0 127.0667197697884,37.03696546138421,0 127.0654330874604,37.03842020263603,0 127.0572593160559,37.04355578913451,0 127.0498707837593,37.03838370906607,0 127.054266060945,37.03416232535104,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SSE_PTK_CD_02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>127.0413386931776,37.03474278763444,0 127.0412324082724,37.0275387731083,0 127.0537443084687,37.02756778899481,0 127.0537899381729,37.03312095301939,0 127.0532473740154,37.03428306717585,0 127.0492058809542,37.03798221468324,0 127.0456061252981,37.03544466619057,0 127.0438028119331,37.03478058034693,0 127.0413386931776,37.03474278763444,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SSE_ONY_CD_01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>127.0605278746439,36.76971779132401,0 127.0601299873631,36.76877854651263,0 127.0599373155932,36.76693414064871,0 127.0599716237569,36.76592169674802,0 127.0608068946097,36.76273356091263,0 127.0629839415533,36.76294664014682,0 127.0652322272324,36.7629534711673,0 127.0650475448265,36.76398706984051,0 127.0642531660493,36.76421241295863,0 127.0641854724725,36.76475044268346,0 127.0639187684978,36.76474551638618,0 127.0639113488801,36.76559270079453,0 127.064878991032,36.76561608736078,0 127.0655601786528,36.76590429560554,0 127.0650143204454,36.76645360616786,0 127.0650751874492,36.76876719588719,0 127.0647600225282,36.77007735700907,0 127.0605278746439,36.76971779132401,0</t>
         </is>
       </c>
     </row>
@@ -6566,7 +6787,1215 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14.6640625" customWidth="1" min="1" max="1"/>
+    <col width="17.5" customWidth="1" min="2" max="2"/>
+    <col width="14.1640625" customWidth="1" min="3" max="3"/>
+    <col width="42.1640625" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="21" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>zone_code</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>effective_from</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>effective_to</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SKH_ICH_OP_01</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>127.4797427,37.2514443,0 127.4797427,37.2500277,0 127.4828987,37.2500277,0 127.4828987,37.2514443,0 127.4797427,37.2514443,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SKH_ICH_OP_02</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>127.4849454900732,37.24696852565402,0 127.4849577805763,37.24804787377957,0 127.4834402050251,37.24804930340976,0 127.4834430926005,37.24697773839749,0 127.4849454900732,37.24696852565402,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SKH_ICH_OP_03</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>127.4798595705619,37.24980238528374,0 127.4798276156388,37.24676972135467,0 127.4817380296342,37.2467803411346,0 127.4817475159931,37.24980517492403,0 127.4798595705619,37.24980238528374,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SKH_ICH_OP_04</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>127.4852091,37.2497203,0 127.4852257,37.2483622,0 127.4871882,37.2483701,0 127.4871756,37.2497296,0 127.4852091,37.2497203,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SKH_ICH_OP_05</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>127.4841102901286,37.2499819551286,0 127.4879200552699,37.24997997851406,0 127.4879330279036,37.25149134619419,0 127.4841022,37.2515,0 127.4841102901286,37.2499819551286,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SKH_ICH_OP_06</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>127.4827095,37.2496922,0 127.4827136,37.2483967,0 127.4850077,37.2483955,0 127.4850164872248,37.24968411315396,0 127.4827095,37.2496922,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SKH_ICH_EX_01</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>2021-06-30</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>127.4841102901286,37.2499819551286,0 127.4879200552699,37.24997997851406,0 127.4879330279036,37.25149134619419,0 127.4841022,37.2515,0 127.4841102901286,37.2499819551286,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SKH_ICH_CD_01</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>127.4792908753239,37.25468493538708,0 127.4786741753453,37.25444924351592,0 127.4772528388912,37.25395564829143,0 127.4767669938143,37.25346355087292,0 127.4760965089844,37.2524207558015,0 127.4754361562875,37.25013297475242,0 127.4755263691511,37.24998272523067,0 127.4761815390762,37.24996768272318,0 127.4762852154837,37.2491772417373,0 127.4766660853097,37.24888413057281,0 127.4770365177835,37.24820942523911,0 127.4770129777922,37.24630386888008,0 127.4783445671774,37.24652078460043,0 127.4794165116467,37.24653038307022,0 127.4797541563503,37.24665384241348,0 127.4823052038301,37.24663760873185,0 127.4826221319934,37.24669367528909,0 127.4826199787886,37.24693028697282,0 127.4839309344984,37.24692849021164,0 127.4851389162666,37.24673774714464,0 127.4857037675637,37.24680396813539,0 127.4864819820665,37.24661121408833,0 127.4878377799842,37.24645368922819,0 127.4878622737257,37.24765802504077,0 127.4887095942767,37.24765852211029,0 127.4887172526127,37.24795890179502,0 127.4909139624968,37.24894757882421,0 127.4906904523238,37.24976641620731,0 127.4901601862512,37.25102843554481,0 127.4886617641543,37.25291476424426,0 127.4869696609773,37.25478884788198,0 127.4861705759206,37.25455007950498,0 127.4853195412984,37.25499405132114,0 127.4845027267799,37.25543761273426,0 127.4841281940734,37.25522463987738,0 127.4797279161993,37.25522397442263,0 127.4792908753239,37.25468493538708,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_OP_01</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>127.4316253,36.6470268,0 127.4278012,36.6470535,0 127.4277877,36.6458126,0 127.4284428,36.6458073,0 127.428441,36.6456247,0 127.4316067,36.6456081,0 127.4316253,36.6470268,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_OP_02</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>127.4236652,36.6485075,0 127.4250183,36.6483869,0 127.4252423,36.6500218,0 127.4238914,36.6501423,0 127.4236652,36.6485075,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_OP_03</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>127.4287742,36.6544496,0 127.4325052,36.6547355,0 127.4323194,36.6563298,0 127.4285806,36.6560474,0 127.4287742,36.6544496,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_OP_04</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>127.4323581,36.6563306,0 127.4325343,36.6547414,0 127.4349417,36.6549244,0 127.4347554,36.6565182,0 127.4323581,36.6563306,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_EX_01</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>127.4314444960006,36.64983218771054,0 127.4338702544078,36.64982696911132,0 127.4338705240823,36.65090889299547,0 127.4314709477459,36.65090531906605,0 127.4314444960006,36.64983218771054,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_EX_02</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>2022-10-01</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>127.4323581,36.6563306,0 127.4325343,36.6547414,0 127.4349417,36.6549244,0 127.4347554,36.6565182,0 127.4323581,36.6563306,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_EX_03</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>127.4301916965771,36.66274946988656,0 127.4272990870079,36.66247998747166,0 127.4278943044712,36.65923800704126,0 127.4306933586569,36.6595070954642,0 127.4301916965771,36.66274946988656,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_CD_01</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>127.4275297354299,36.65233372032262,0 127.4263057730211,36.65185408401877,0 127.4262935535888,36.65122515869427,0 127.4275256456034,36.65122133567544,0 127.4275201588123,36.64961054877304,0 127.4312464208049,36.64960916510265,0 127.4312470904888,36.64952629302427,0 127.4351002158643,36.64950044912582,0 127.435166824625,36.65359448360476,0 127.432862488071,36.65359823906715,0 127.4316649289962,36.65337928541467,0 127.4308305599157,36.65296363320886,0 127.4288246715552,36.65263268339037,0 127.4275297354299,36.65233372032262,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_CD_02</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>127.4260432086972,36.65176170137349,0 127.4248531681613,36.65127349565639,0 127.4237537290272,36.65063059263603,0 127.4234767236715,36.65009942631145,0 127.4232265303528,36.64810824397203,0 127.4247733956071,36.64798844700252,0 127.4255746104511,36.64780770534722,0 127.4260432086972,36.65176170137349,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_CD_03</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>127.4317942851492,36.64759990559355,0 127.4275552059397,36.64762560914508,0 127.4274902029552,36.64587102656827,0 127.4294903446101,36.64501362772035,0 127.4317576818901,36.64466362443578,0 127.4317942851492,36.64759990559355,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_CD_04</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>127.4292728903329,36.65737585583252,0 127.4273960610812,36.65679768320321,0 127.4282675369856,36.6554496975609,0 127.4284050618595,36.65469966598357,0 127.4282398485941,36.65293596566627,0 127.4304563399528,36.65307861551903,0 127.4316145244017,36.65366103982478,0 127.4326545386969,36.65382547046487,0 127.4350916090492,36.65392998807685,0 127.4352735323493,36.65785267344271,0 127.4292728903329,36.65737585583252,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SKH_CJJ_CD_05</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>127.4243211838829,36.6632598487266,0 127.424011351887,36.65991970480072,0 127.4229741451245,36.65607422634487,0 127.4244942262898,36.65536905146344,0 127.4257468499067,36.65639926020843,0 127.4267895578782,36.65700917768972,0 127.4282817570568,36.65755430873217,0 127.4297234332019,36.6578268621073,0 127.4353019051501,36.65834157696911,0 127.4356995447989,36.66481575781614,0 127.433912758689,36.66409712773648,0 127.4282703545717,36.66376686338138,0 127.4243211838829,36.6632598487266,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SKH_YIN_EX_01</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>2025-02-24</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>127.3179076794612,37.15878095033005,0 127.3171855420929,37.1569370023885,0 127.3245611539538,37.15531271600427,0 127.3252504596098,37.15718533783891,0 127.3179076794612,37.15878095033005,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SKH_YIN_CD_01</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>2025-02-24</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>127.3165991989156,37.15980583693546,0 127.3128009723789,37.14835919575778,0 127.311076347084,37.14547863343643,0 127.3102408044489,37.14303692870982,0 127.3208615727544,37.14061591456515,0 127.3220561267111,37.1417979786553,0 127.3247735631805,37.14850423312373,0 127.324982600008,37.15064631017324,0 127.3266053447182,37.15485998175167,0 127.3279031725835,37.15572439755587,0 127.328670071381,37.15778146758801,0 127.3183489938163,37.16020717025311,0 127.3165991989156,37.15980583693546,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SSE_GHG_OP_01</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>127.0848247936377,37.22976441277449,0 127.084816697626,37.22874171437098,0 127.0871417626563,37.2287586132593,0 127.0871522519888,37.22976607272437,0 127.0848247936377,37.22976441277449,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SSE_GHG_OP_02</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>127.0848212251696,37.22745084800816,0 127.0871134773173,37.22745989465779,0 127.0871368314815,37.22853523488989,0 127.0848331,37.2285342,0 127.0848212251696,37.22745084800816,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SSE_GHG_OP_03</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>127.0848455,37.2258866,0 127.0870337752034,37.22588140105419,0 127.0870406255941,37.2271457994231,0 127.0848498752152,37.22713771127859,0 127.0848455,37.2258866,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SSE_GHG_CD_01</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>127.083461691631,37.22989691093171,0 127.083042227891,37.22951575495898,0 127.0829522524925,37.22638055251159,0 127.0844632219606,37.22638940835161,0 127.0844822059877,37.22570474903128,0 127.0887076667388,37.22570338865468,0 127.089052454588,37.22595566548927,0 127.089026146627,37.22718421375711,0 127.0895887134091,37.22719165032877,0 127.0891868539899,37.22816160042641,0 127.0887849945707,37.22913155052407,0 127.0880244523491,37.22991225379975,0 127.083461691631,37.22989691093171,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SSE_HWA_OP_01</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>127.0619712,37.2212668,0 127.0628744,37.2202075,0 127.062759,37.220137,0 127.0629513,37.2199471,0 127.0651172,37.2211755,0 127.0650018,37.221295,0 127.0651633,37.2213899,0 127.064971,37.2215707,0 127.0650864,37.2216411,0 127.0642293,37.2225625,0 127.0619712,37.2212668,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SSE_HWA_OP_02</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>127.064106,37.218391,0 127.0661072,37.219557,0 127.0658884,37.2197978,0 127.0660833,37.2199086,0 127.0656258,37.2204251,0 127.0654468,37.2203142,0 127.0651216,37.2206677,0 127.0631192,37.2195397,0 127.064106,37.218391,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SSE_HWA_OP_03</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>127.0692329,37.2173087,0 127.0674072,37.2169974,0 127.0679785,37.2145846,0 127.0698561,37.2149052,0 127.0692329,37.2173087,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SSE_HWA_OP_04</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>127.0661214,37.2124709,0 127.0703728,37.2131454,0 127.0701773,37.2140141,0 127.0705154,37.2140702,0 127.070375,37.2145903,0 127.0658359,37.2138277,0 127.0661214,37.2124709,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SSE_HWA_OP_05</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>127.0714076,37.2149811,0 127.0759209,37.2157293,0 127.0755203,37.2174274,0 127.0709793,37.2167086,0 127.0714076,37.2149811,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SSE_HWA_OP_06</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>2020-02-01</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>127.0718011,37.2133492,0 127.0753872,37.2139181,0 127.0751035,37.2151765,0 127.0715272,37.2146116,0 127.0718011,37.2133492,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SSE_HWA_EX_01</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-31</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>127.0718011,37.2133492,0 127.0753872,37.2139181,0 127.0751035,37.2151765,0 127.0715272,37.2146116,0 127.0718011,37.2133492,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SSE_HWA_CD_01</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>127.0604088113161,37.22131882984505,0 127.0615807830927,37.22041598662344,0 127.0630934084169,37.21750233768811,0 127.0634913563929,37.21689581411416,0 127.0648657301476,37.21768520734643,0 127.0645369158691,37.21804783507638,0 127.0649234166045,37.21824765192734,0 127.0647277837963,37.21847858521478,0 127.0662831589923,37.21938670995086,0 127.06664594273,37.21885044069479,0 127.0670258100668,37.2180123534205,0 127.0670166258656,37.21713827335517,0 127.0674025178071,37.2155538216505,0 127.0667276391382,37.21500375126403,0 127.0655461123071,37.2149879687613,0 127.0648952488986,37.21559495354837,0 127.0634374596184,37.21535848732494,0 127.0642118961364,37.2123743909837,0 127.0651782203331,37.21208702120425,0 127.0677572511424,37.21194828414612,0 127.0705415107046,37.21031086343675,0 127.0728251102545,37.2120405976308,0 127.0781759625584,37.2149215297925,0 127.0774851858635,37.21729625905924,0 127.076012950966,37.22023406713998,0 127.0730025425854,37.21894843108969,0 127.0718544566005,37.21858037365727,0 127.0695738141374,37.21824888550046,0 127.0690641747031,37.21989668149228,0 127.0678519558422,37.21967489336973,0 127.0678501450078,37.21927789628356,0 127.0668359627562,37.21905080170365,0 127.0665419684045,37.21945597062771,0 127.065715293898,37.221067494351,0 127.0650135511269,37.22274342329509,0 127.0649907298155,37.22317211827212,0 127.0646802506171,37.2231710187238,0 127.0643725197762,37.22354909864806,0 127.0632761594175,37.22369709565476,0 127.0619533378606,37.22289446612139,0 127.0604088113161,37.22131882984505,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SSE_PTK_OP_01</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>127.0546191,37.0375397,0 127.0606411,37.037526,0 127.0606393,37.0393664,0 127.0545883,37.0393679,0 127.0546191,37.0375397,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SSE_PTK_OP_02</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>2020-08-30</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>127.0627462,37.0357638,0 127.0568884,37.0357886,0 127.056883,37.0339202,0 127.0627513,37.0339331,0 127.0627462,37.0357638,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SSE_PTK_OP_03</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>127.0563073,37.0359889,0 127.0544513,37.0359978,0 127.0544292,37.0343399,0 127.0563183,37.0343575,0 127.0563073,37.0359889,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SSE_PTK_OP_04</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>2022-09-07</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>127.0639785,37.0334678,0 127.0567843,37.033462,0 127.0568184,37.0315637,0 127.0639849,37.0315702,0 127.0639785,37.0334678,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SSE_PTK_OAE_01</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>127.0640161,37.0297022,0 127.0567316,37.0297043,0 127.0567687,37.027796,0 127.0640161,37.0278605,0 127.0640161,37.0297022,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SSE_PTK_EX_01</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>2020-08-29</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>127.0627462,37.0357638,0 127.0568884,37.0357886,0 127.056883,37.0339202,0 127.0627513,37.0339331,0 127.0627462,37.0357638,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SSE_PTK_EX_02</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>2021-06-30</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>127.0563073,37.0359889,0 127.0544513,37.0359978,0 127.0544292,37.0343399,0 127.0563183,37.0343575,0 127.0563073,37.0359889,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SSE_PTK_EX_03</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>2022-09-06</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>127.0639785,37.0334678,0 127.0567843,37.033462,0 127.0568184,37.0315637,0 127.0639849,37.0315702,0 127.0639785,37.0334678,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SSE_PTK_EX_04</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>2021-10-18</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>127.0640161,37.0297022,0 127.0567316,37.0297043,0 127.0567687,37.027796,0 127.0640161,37.0278605,0 127.0640161,37.0297022,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SSE_PTK_EX_05</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>2022-07-01</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>127.0449749659105,37.0300120145176,0 127.0449866280244,37.02790717862602,0 127.0519163975255,37.02786910386619,0 127.0519054389011,37.03004190658875,0 127.0449749659105,37.0300120145176,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SSE_PTK_EX_06</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>127.0450255702362,37.0338147847025,0 127.0450607984398,37.03182733203584,0 127.0519865,37.0318094,0 127.0519865,37.0338084,0 127.0450255702362,37.0338147847025,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SSE_PTK_CD_01</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>127.054266060945,37.03416232535104,0 127.0543122205523,37.02756427257659,0 127.0681249737192,37.0275595754502,0 127.0674879668247,37.03507496714188,0 127.0667197697884,37.03696546138421,0 127.0654330874604,37.03842020263603,0 127.0572593160559,37.04355578913451,0 127.0498707837593,37.03838370906607,0 127.054266060945,37.03416232535104,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SSE_PTK_CD_02</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>127.0413386931776,37.03474278763444,0 127.0412324082724,37.0275387731083,0 127.0537443084687,37.02756778899481,0 127.0537899381729,37.03312095301939,0 127.0532473740154,37.03428306717585,0 127.0492058809542,37.03798221468324,0 127.0456061252981,37.03544466619057,0 127.0438028119331,37.03478058034693,0 127.0413386931776,37.03474278763444,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SSE_ONY_OP_01</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>127.0614227,36.7672679,0 127.0614119,36.7663013,0 127.0623034,36.7662956,0 127.0623213,36.7672708,0 127.0614227,36.7672679,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SSE_ONY_OP_02</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>127.061431,36.7660969,0 127.0614287,36.7651813,0 127.0623252,36.7651787,0 127.0623283,36.7660925,0 127.061431,36.7660969,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SSE_ONY_OP_03</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>127.0625218,36.7660891,0 127.0625218,36.7651691,0 127.0634068,36.7651727,0 127.0634181,36.7660891,0 127.0625218,36.7660891,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>SSE_ONY_OP_04</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>127.0617674,36.7649643,0 127.0617721,36.7639231,0 127.0633897,36.7639243,0 127.0634044,36.7649679,0 127.0617674,36.7649643,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SSE_ONY_EX_01</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>127.0621781,36.7637454,0 127.0621964,36.7630197,0 127.0648637,36.7630455,0 127.0648544,36.7637586,0 127.0621781,36.7637454,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>SSE_ONY_CD_01</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>127.0605278746439,36.76971779132401,0 127.0601299873631,36.76877854651263,0 127.0599373155932,36.76693414064871,0 127.0599716237569,36.76592169674802,0 127.0608068946097,36.76273356091263,0 127.0629839415533,36.76294664014682,0 127.0652322272324,36.7629534711673,0 127.0650475448265,36.76398706984051,0 127.0642531660493,36.76421241295863,0 127.0641854724725,36.76475044268346,0 127.0639187684978,36.76474551638618,0 127.0639113488801,36.76559270079453,0 127.064878991032,36.76561608736078,0 127.0655601786528,36.76590429560554,0 127.0650143204454,36.76645360616786,0 127.0650751874492,36.76876719588719,0 127.0647600225282,36.77007735700907,0 127.0605278746439,36.76971779132401,0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6578,8 +8007,9 @@
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="42.1640625" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="13.5" customWidth="1" min="6" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7528,11 +8958,12 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7556,6 +8987,7 @@
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="18" customWidth="1" min="18" max="18"/>
     <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="13.5" customWidth="1" min="20" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8952,10 +10384,8 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="H15" t="n">
+        <v>6</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -9437,10 +10867,8 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+      <c r="H20" t="n">
+        <v>15</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -9534,10 +10962,8 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="H21" t="n">
+        <v>16</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -10954,444 +12380,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>zone_code</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>polygon</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>SKH_ICH_OP_03</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>127.4841047,37.2500254,0 127.487888,37.250039,0 127.487873,37.251528,0 127.4841022,37.2515,0 127.4841047,37.2500254,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>SKH_ICH_OP_02</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>127.4796695,37.2497298,0 127.4797232,37.2466564,0 127.4813396,37.2466588,0 127.481358,37.249322,0 127.481362,37.249743,0 127.4796695,37.2497298,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>SKH_ICH_OP_01</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>127.4827095,37.2496922,0 127.4827136,37.2483967,0 127.4850077,37.2483955,0 127.484998,37.2494433,0 127.4847748,37.2494416,0 127.4847676,37.2496922,0 127.4827095,37.2496922,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>SKH_ICH_OP_04</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>127.4797427,37.2514443,0 127.4797427,37.2500277,0 127.4828987,37.2500277,0 127.4828987,37.2514443,0 127.4797427,37.2514443,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>SKH_ICH_OP_06</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>127.4852091,37.2497203,0 127.4852257,37.2483622,0 127.4871882,37.2483701,0 127.4871756,37.2497296,0 127.4852091,37.2497203,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>SKH_ICH_OP_05</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>127.484975,37.2469548,0 127.4849693,37.2480944,0 127.4838393,37.2481222,0 127.4838468,37.2469365,0 127.484975,37.2469548,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>SKH_CJJ_EX_01</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>127.4315085,36.6499593,0 127.4324041,36.6499515,0 127.4324041,36.6498944,0 127.4328465,36.649891,0 127.4328474,36.6499508,0 127.4339363,36.6499452,0 127.4339443,36.6509217,0 127.4329256,36.6509264,0 127.4329241,36.651076,0 127.4325161,36.6510795,0 127.4325161,36.6509297,0 127.4315277,36.6509344,0 127.4315085,36.6499593,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>SKH_CJJ_OP_01</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>127.4236652,36.6485075,0 127.4250183,36.6483869,0 127.4252423,36.6500218,0 127.4238914,36.6501423,0 127.4236652,36.6485075,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>SKH_CJJ_OP_02</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>127.4316253,36.6470268,0 127.4278012,36.6470535,0 127.4277877,36.6458126,0 127.4284428,36.6458073,0 127.428441,36.6456247,0 127.4316067,36.6456081,0 127.4316253,36.6470268,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>SKH_CJJ_OP_03</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>127.4287742,36.6544496,0 127.4325052,36.6547355,0 127.4323194,36.6563298,0 127.4285806,36.6560474,0 127.4287742,36.6544496,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>SKH_CJJ_OP_04</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>127.4323581,36.6563306,0 127.4325343,36.6547414,0 127.4349417,36.6549244,0 127.4347554,36.6565182,0 127.4323581,36.6563306,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>SKH_CJJ_EX_02</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>127.4306473,36.6596684,0 127.430228,36.6625682,0 127.427628,36.662326,0 127.4280473,36.659406,0 127.4306473,36.6596684,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>SKH_YIN_EX_01</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>127.3186406,37.1599045,0 127.3172996,37.1599175,0 127.3162805,37.1594805,0 127.3139929,37.1527064,0 127.3141608,37.1514519,0 127.313207,37.1486771,0 127.3111075,37.1454116,0 127.3221344,37.1429897,0 127.3265194,37.1551081,0 127.3276958,37.1555952,0 127.3284789,37.1576138,0 127.3186406,37.1599045,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>SSE_GHG_OP_01</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>127.0848557,37.2296894,0 127.0848582,37.2287584,0 127.0872233,37.2287594,0 127.0872251,37.2296801,0 127.0848557,37.2296894,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>SSE_GHG_OP_02</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>127.084815,37.2274814,0 127.0872511,37.2274429,0 127.0872783,37.2284885,0 127.0848331,37.2285342,0 127.084815,37.2274814,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>SSE_GHG_OP_03</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>127.0848455,37.2258866,0 127.08698,37.2258735,0 127.0870488,37.2271066,0 127.0848946,37.2271378,0 127.0848455,37.2258866,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>SSE_HWA_OP_01</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>127.0619712,37.2212668,0 127.0628744,37.2202075,0 127.062759,37.220137,0 127.0629513,37.2199471,0 127.0651172,37.2211755,0 127.0650018,37.221295,0 127.0651633,37.2213899,0 127.064971,37.2215707,0 127.0650864,37.2216411,0 127.0642293,37.2225625,0 127.0619712,37.2212668,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>SSE_HWA_OP_02</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>127.064106,37.218391,0 127.0661072,37.219557,0 127.0658884,37.2197978,0 127.0660833,37.2199086,0 127.0656258,37.2204251,0 127.0654468,37.2203142,0 127.0651216,37.2206677,0 127.0631192,37.2195397,0 127.064106,37.218391,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>SSE_HWA_OP_03</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>127.0692329,37.2173087,0 127.0674072,37.2169974,0 127.0679785,37.2145846,0 127.0698561,37.2149052,0 127.0692329,37.2173087,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>SSE_HWA_OP_04</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>127.0661214,37.2124709,0 127.0703728,37.2131454,0 127.0701773,37.2140141,0 127.0705154,37.2140702,0 127.070375,37.2145903,0 127.0658359,37.2138277,0 127.0661214,37.2124709,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>SSE_HWA_OP_05</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>127.0714076,37.2149811,0 127.0759209,37.2157293,0 127.0755203,37.2174274,0 127.0709793,37.2167086,0 127.0714076,37.2149811,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>SSE_HWA_OP_06</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>127.0718011,37.2133492,0 127.0753872,37.2139181,0 127.0751035,37.2151765,0 127.0715272,37.2146116,0 127.0718011,37.2133492,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>SSE_PTK_OP_01</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>127.0546191,37.0375397,0 127.0606411,37.037526,0 127.0606393,37.0393664,0 127.0545883,37.0393679,0 127.0546191,37.0375397,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>SSE_PTK_OP_02</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>127.0627462,37.0357638,0 127.0568884,37.0357886,0 127.056883,37.0339202,0 127.0627513,37.0339331,0 127.0627462,37.0357638,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>SSE_PTK_OP_03</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>127.0639785,37.0334678,0 127.0567843,37.033462,0 127.0568184,37.0315637,0 127.0639849,37.0315702,0 127.0639785,37.0334678,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>SSE_PTK_OP_04</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>127.0640161,37.0297022,0 127.0567316,37.0297043,0 127.0567687,37.027796,0 127.0640161,37.0278605,0 127.0640161,37.0297022,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>SSE_PTK_EX_01</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>127.0451099,37.0338391,0 127.0451291,37.0318094,0 127.0519865,37.0318094,0 127.0519865,37.0338084,0 127.0451099,37.0338391,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>SSE_PTK_EX_02</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>127.0446729,37.0301421,0 127.0446851,37.0277274,0 127.0526079,37.0277079,0 127.0526447,37.0301519,0 127.0446729,37.0301421,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>SSE_PTK_OP_05</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>127.0563073,37.0359889,0 127.0544513,37.0359978,0 127.0544292,37.0343399,0 127.0563183,37.0343575,0 127.0563073,37.0359889,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>SSE_ONY_OP_01</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>127.0614227,36.7672679,0 127.0614119,36.7663013,0 127.0623034,36.7662956,0 127.0623213,36.7672708,0 127.0614227,36.7672679,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>SSE_ONY_OP_02</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>127.061431,36.7660969,0 127.0614287,36.7651813,0 127.0623252,36.7651787,0 127.0623283,36.7660925,0 127.061431,36.7660969,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>SSE_ONY_OP_03</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>127.0625218,36.7660891,0 127.0625218,36.7651691,0 127.0634068,36.7651727,0 127.0634181,36.7660891,0 127.0625218,36.7660891,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>SSE_ONY_OP_04</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>127.0617674,36.7649643,0 127.0617721,36.7639231,0 127.0633897,36.7639243,0 127.0634044,36.7649679,0 127.0617674,36.7649643,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>SSE_ONY_EX_01</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>127.0621781,36.7637454,0 127.0621964,36.7630197,0 127.0648637,36.7630455,0 127.0648544,36.7637586,0 127.0621781,36.7637454,0</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>